<commit_message>
Add config engine, transfers & repair features
Introduce v2 features: add a ConfigEngine (config.json) for custom departments/types/conditions and wire it into the JS API. Extend ExcelEngine and API to support Transfer History, asset transfers, improved replacement/repair handling, automatic condition updates, and transfer/history reads; add Transfer History column and Config sheet handling and robust migration/cleanup logic. Add a portable app builder (INSTALL_ON_NEW_PC scripts + README) and update logging/action tags. Update UI title and styling (ui.html) and bump start.bat/main metadata and window sizing. README updated to document v2 features, security notes, and portable install instructions.
</commit_message>
<xml_diff>
--- a/ICT_MASTER.xlsx
+++ b/ICT_MASTER.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7695" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="History" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Replacements" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Ink" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Audit Log" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="History" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Replacements" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ink" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Log" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Corbel"/>
       <charset val="134"/>
@@ -34,8 +35,13 @@
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -45,6 +51,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F2937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F2937"/>
       </patternFill>
     </fill>
   </fills>
@@ -60,10 +71,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -396,7 +411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O423"/>
+  <dimension ref="A1:P423"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="1" min="1" max="2"/>
@@ -490,6 +505,11 @@
           <t>Remarks</t>
         </is>
       </c>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>Transfer History</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -16263,7 +16283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="21.95" customHeight="1" s="1">
@@ -16338,7 +16358,38 @@
       <c r="G2" t="n">
         <v>1</v>
       </c>
-      <c r="H2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-30 05:35:19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BK</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>restock</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16351,7 +16402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="21.95" customHeight="1" s="1">
@@ -16398,6 +16449,54 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-30 05:35:19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>INK</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Ink restock: 1x Black (BK)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ICT Manager</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" s="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 'by' tracking and transfer authorisation
Persist and surface who authorised/performed actions across the app. Added a 'by' field to history reads/writes and updated ExcelEngine and Api method signatures to accept an optional by (defaulting to "ICT Manager"). UI additions include an Asset Report section, transfer "Authorised By" input, repair workflow (banner, mark-as-repaired shortcut, cost/technician fields), custom dropdowns supporting an "Other / type custom" entry, and visual cues for items needing repair. Also updated chart rendering (doughnut percentages), session/ PIN UX, and various helper functions (fillSelWithCustom, showCustomInput, getSelVal/setSelVal). The MASTER Excel workbook was updated accordingly to store the new column.
</commit_message>
<xml_diff>
--- a/ICT_MASTER.xlsx
+++ b/ICT_MASTER.xlsx
@@ -16283,7 +16283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="21.95" customHeight="1" s="1">
@@ -16358,38 +16358,6 @@
       <c r="G2" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-05-30 05:35:19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>BK</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>restock</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16402,7 +16370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="21.95" customHeight="1" s="1">
@@ -16444,28 +16412,6 @@
         </is>
       </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>ICT Manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-05-30 05:35:19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>INK</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Ink restock: 1x Black (BK)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
         <is>
           <t>ICT Manager</t>
         </is>

</xml_diff>